<commit_message>
refactor(bridge): inline chip crew effects and source slots from Core Excel
</commit_message>
<xml_diff>
--- a/tools/data_source/module_data.xlsx
+++ b/tools/data_source/module_data.xlsx
@@ -921,63 +921,86 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
-  <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="4.25" customWidth="1"/>
-    <col min="6" max="7" width="48" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>size</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>energy_cost</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>texture_path</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>crew_slots</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>chip_slots</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>core_bridge</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>舰桥</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>飞船核心区域。核心模块被击毁时，飞船判定为沉没。</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2x2</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>res://data/assets/modules/core_bridge.png</t>
+        </is>
+      </c>
+      <c r="G2">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E2" s="2">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" ht="18" customHeight="1"/>
+      <c r="H2">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>